<commit_message>
Refresh earnings tracker styling and add Engaged Views column
Switches to a cleaner navy/steel-blue palette instead of the bright
red/yellow scheme, and adds an Engaged Views column (monetized
playbacks) so RPM and the Average RPM summary are calculated against
engaged views rather than total views.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S454NQMsGhA62HZVzwmSTo
</commit_message>
<xml_diff>
--- a/YouTube_Earnings_Tracker.xlsx
+++ b/YouTube_Earnings_Tracker.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="166" formatCode="$#,##0.00"/>
     <numFmt numFmtId="167" formatCode="$0.00"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,71 +31,66 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="20"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="00595959"/>
+      <color rgb="006B7280"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00000000"/>
+      <color rgb="001F2A44"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <color rgb="000000FF"/>
+      <name val="Calibri"/>
+      <color rgb="0015417E"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <color rgb="00000000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="13"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00000000"/>
+      <color rgb="001F2A44"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00CC0000"/>
+      <color rgb="001E5B32"/>
       <sz val="13"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="007F7F7F"/>
-      <sz val="9"/>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E5B32"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -104,27 +99,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00282828"/>
+        <fgColor rgb="001F2A44"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FF0000"/>
+        <fgColor rgb="002E5A88"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CC0000"/>
+        <fgColor rgb="00F4F6F8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF9C4"/>
+        <fgColor rgb="00EAF2FB"/>
       </patternFill>
     </fill>
     <fill>
@@ -134,12 +124,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
+        <fgColor rgb="00EDEFF2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00E3F0E6"/>
       </patternFill>
     </fill>
   </fills>
@@ -153,23 +143,23 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00D9DEE4"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00D9DEE4"/>
       </right>
       <top style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00D9DEE4"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00D9DEE4"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -180,44 +170,48 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -585,17 +579,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1">
+    <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>YouTube Earnings Tracker</t>
@@ -613,12 +608,12 @@
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Legend: Yellow cells = enter your monthly numbers  |  Blue text = your input  |  Black text = auto-calculated formula</t>
+          <t>Legend:  Pale blue cells = enter your monthly numbers   |   Blue text = your input   |   Navy text = auto-calculated formula</t>
         </is>
       </c>
     </row>
     <row r="5" ht="6" customHeight="1"/>
-    <row r="6" ht="22" customHeight="1">
+    <row r="6" ht="30" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Month</t>
@@ -636,10 +631,15 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
+          <t>Engaged Views</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
           <t>Earnings ($)</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>RPM ($)</t>
         </is>
@@ -655,13 +655,16 @@
         <v>8</v>
       </c>
       <c r="C7" s="6" t="n">
+        <v>60000</v>
+      </c>
+      <c r="D7" s="6" t="n">
         <v>50000</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="E7" s="7" t="n">
         <v>200</v>
       </c>
-      <c r="E7" s="8">
-        <f>IFERROR(D7/C7*1000,0)</f>
+      <c r="F7" s="8">
+        <f>IFERROR(E7/D7*1000,0)</f>
         <v>4</v>
       </c>
     </row>
@@ -675,13 +678,16 @@
         <v>10</v>
       </c>
       <c r="C8" s="6" t="n">
+        <v>95000</v>
+      </c>
+      <c r="D8" s="6" t="n">
         <v>80000</v>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="E8" s="7" t="n">
         <v>400</v>
       </c>
-      <c r="E8" s="10">
-        <f>IFERROR(D8/C8*1000,0)</f>
+      <c r="F8" s="10">
+        <f>IFERROR(E8/D8*1000,0)</f>
         <v>5</v>
       </c>
     </row>
@@ -693,9 +699,10 @@
       </c>
       <c r="B9" s="6" t="n"/>
       <c r="C9" s="6" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="8">
-        <f>IFERROR(D9/C9*1000,0)</f>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="8">
+        <f>IFERROR(E9/D9*1000,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -707,9 +714,10 @@
       </c>
       <c r="B10" s="6" t="n"/>
       <c r="C10" s="6" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="10">
-        <f>IFERROR(D10/C10*1000,0)</f>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="10">
+        <f>IFERROR(E10/D10*1000,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -721,9 +729,10 @@
       </c>
       <c r="B11" s="6" t="n"/>
       <c r="C11" s="6" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="8">
-        <f>IFERROR(D11/C11*1000,0)</f>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="8">
+        <f>IFERROR(E11/D11*1000,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -735,9 +744,10 @@
       </c>
       <c r="B12" s="6" t="n"/>
       <c r="C12" s="6" t="n"/>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="10">
-        <f>IFERROR(D12/C12*1000,0)</f>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="10">
+        <f>IFERROR(E12/D12*1000,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -749,9 +759,10 @@
       </c>
       <c r="B13" s="6" t="n"/>
       <c r="C13" s="6" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="8">
-        <f>IFERROR(D13/C13*1000,0)</f>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="8">
+        <f>IFERROR(E13/D13*1000,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -763,9 +774,10 @@
       </c>
       <c r="B14" s="6" t="n"/>
       <c r="C14" s="6" t="n"/>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="10">
-        <f>IFERROR(D14/C14*1000,0)</f>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="10">
+        <f>IFERROR(E14/D14*1000,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -777,9 +789,10 @@
       </c>
       <c r="B15" s="6" t="n"/>
       <c r="C15" s="6" t="n"/>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="8">
-        <f>IFERROR(D15/C15*1000,0)</f>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="7" t="n"/>
+      <c r="F15" s="8">
+        <f>IFERROR(E15/D15*1000,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -791,9 +804,10 @@
       </c>
       <c r="B16" s="6" t="n"/>
       <c r="C16" s="6" t="n"/>
-      <c r="D16" s="7" t="n"/>
-      <c r="E16" s="10">
-        <f>IFERROR(D16/C16*1000,0)</f>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="10">
+        <f>IFERROR(E16/D16*1000,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -814,7 +828,8 @@
       <c r="B19" s="13" t="n"/>
       <c r="C19" s="13" t="n"/>
       <c r="D19" s="13" t="n"/>
-      <c r="E19" s="14">
+      <c r="E19" s="13" t="n"/>
+      <c r="F19" s="14">
         <f>SUM(B7:B16)</f>
         <v>18</v>
       </c>
@@ -828,57 +843,76 @@
       <c r="B20" s="13" t="n"/>
       <c r="C20" s="13" t="n"/>
       <c r="D20" s="13" t="n"/>
-      <c r="E20" s="14">
+      <c r="E20" s="13" t="n"/>
+      <c r="F20" s="14">
         <f>SUM(C7:C16)</f>
-        <v>130000</v>
+        <v>155000</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>Total Earnings</t>
+          <t>Total Engaged Views</t>
         </is>
       </c>
       <c r="B21" s="13" t="n"/>
       <c r="C21" s="13" t="n"/>
       <c r="D21" s="13" t="n"/>
-      <c r="E21" s="15">
+      <c r="E21" s="13" t="n"/>
+      <c r="F21" s="14">
         <f>SUM(D7:D16)</f>
+        <v>130000</v>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>Total Earnings</t>
+        </is>
+      </c>
+      <c r="B22" s="16" t="n"/>
+      <c r="C22" s="16" t="n"/>
+      <c r="D22" s="16" t="n"/>
+      <c r="E22" s="16" t="n"/>
+      <c r="F22" s="17">
+        <f>SUM(E7:E16)</f>
         <v>600</v>
       </c>
     </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="12" t="inlineStr">
-        <is>
-          <t>Average RPM (Total Earnings ÷ Total Views × 1000)</t>
-        </is>
-      </c>
-      <c r="B22" s="13" t="n"/>
-      <c r="C22" s="13" t="n"/>
-      <c r="D22" s="13" t="n"/>
-      <c r="E22" s="16">
-        <f>IFERROR(E21/E20*1000,0)</f>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>Average RPM (Total Earnings ÷ Total Engaged Views × 1000)</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="n"/>
+      <c r="C23" s="13" t="n"/>
+      <c r="D23" s="13" t="n"/>
+      <c r="E23" s="13" t="n"/>
+      <c r="F23" s="18">
+        <f>IFERROR(F22/F21*1000,0)</f>
         <v>4.6153846153846154</v>
       </c>
     </row>
-    <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="17" t="inlineStr">
-        <is>
-          <t>Note: June and July 2026 are pre-filled with sample figures ($200 and $400 earnings) to illustrate how the Summary totals your data. Replace them with your real numbers from YouTube Studio &gt; Analytics &gt; Revenue, and fill in the remaining months as they happen.</t>
+    <row r="25" ht="42" customHeight="1">
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>Note: "Engaged Views" are the monetized playbacks your revenue is actually paid on (YouTube Studio &gt; Analytics &gt; Revenue &gt; Playback-based CPM), which is why RPM and the Average RPM below are calculated against Engaged Views, not total Views. June and July 2026 are pre-filled with sample figures ($200 and $400 earnings) to show how the Summary adds up to $600 — replace them with your real numbers and fill in the remaining months as they happen.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A24:E24"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="A18:E18"/>
+  <mergeCells count="10">
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="A25:F25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Split earnings tracker into Shorts and Long-Form Videos sections
Adds Shorts Published / Long-form Videos Published as separate counts,
a new Long Views column for long-form videos, and a dedicated RPM per
content type: Shorts RPM uses Engaged Views, Long-Form RPM uses total
Long Views (every long-form view is monetized). Total Earnings per row
and in the Summary is now Shorts earnings + Long-form earnings.

June 2026 is filled in with the user's real reported figures (Shorts:
15 published, 1.1M views, 606.7K engaged, $146.81 earned; Long-form:
1 published, 31.6K views, $59.84 earned — $206.65 combined).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S454NQMsGhA62HZVzwmSTo
</commit_message>
<xml_diff>
--- a/YouTube_Earnings_Tracker.xlsx
+++ b/YouTube_Earnings_Tracker.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="166" formatCode="$#,##0.00"/>
     <numFmt numFmtId="167" formatCode="$0.00"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,6 +57,12 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="001F2A44"/>
       <sz val="10"/>
     </font>
@@ -74,23 +80,29 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001F2A44"/>
-      <sz val="11"/>
+      <color rgb="002E5A88"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="005B7C99"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001E5B32"/>
-      <sz val="13"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001E5B32"/>
-      <sz val="11"/>
+      <sz val="14"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +117,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002E5A88"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005B7C99"/>
       </patternFill>
     </fill>
     <fill>
@@ -124,6 +141,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00DCE4EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00EDEFF2"/>
       </patternFill>
     </fill>
@@ -133,7 +155,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -155,11 +177,25 @@
         <color rgb="00D9DEE4"/>
       </bottom>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="00AAB6C2"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9DEE4"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9DEE4"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9DEE4"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -170,45 +206,84 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="12" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -579,15 +654,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -608,311 +688,635 @@
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Legend:  Pale blue cells = enter your monthly numbers   |   Blue text = your input   |   Navy text = auto-calculated formula</t>
+          <t>Legend:  Pale blue cells = enter your monthly numbers   |   Blue text = your input   |   Navy text = auto-calculated formula   |   Shorts RPM uses Engaged Views, Long-form RPM uses total Long Views (you earn on every long-form view)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="6" customHeight="1"/>
-    <row r="6" ht="30" customHeight="1">
+    <row r="6" ht="20" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>SHORTS</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>LONG-FORM VIDEOS</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="6" t="n"/>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>Total Earnings ($)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="6" t="n"/>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Shorts Published</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Views</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Engaged Views</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>Earnings ($)</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>RPM ($)</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
         <is>
           <t>Videos Published</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Views</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Engaged Views</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="H7" s="11" t="inlineStr">
+        <is>
+          <t>Long Views</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="inlineStr">
         <is>
           <t>Earnings ($)</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="J7" s="11" t="inlineStr">
         <is>
           <t>RPM ($)</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="K7" s="12" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>June 2026</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>60000</v>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>50000</v>
-      </c>
-      <c r="E7" s="7" t="n">
-        <v>200</v>
-      </c>
-      <c r="F7" s="8">
-        <f>IFERROR(E7/D7*1000,0)</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="B8" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>1100000</v>
+      </c>
+      <c r="D8" s="14" t="n">
+        <v>606700</v>
+      </c>
+      <c r="E8" s="15" t="n">
+        <v>146.81</v>
+      </c>
+      <c r="F8" s="16">
+        <f>IFERROR(E8/D8*1000,0)</f>
+        <v>0.24198120982363605</v>
+      </c>
+      <c r="G8" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="14" t="n">
+        <v>31600</v>
+      </c>
+      <c r="I8" s="15" t="n">
+        <v>59.84</v>
+      </c>
+      <c r="J8" s="16">
+        <f>IFERROR(I8/H8*1000,0)</f>
+        <v>1.8936708860759495</v>
+      </c>
+      <c r="K8" s="18">
+        <f>E8+I8</f>
+        <v>206.65</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>July 2026</t>
         </is>
       </c>
-      <c r="B8" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>95000</v>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>80000</v>
-      </c>
-      <c r="E8" s="7" t="n">
-        <v>400</v>
-      </c>
-      <c r="F8" s="10">
-        <f>IFERROR(E8/D8*1000,0)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="B9" s="14" t="n"/>
+      <c r="C9" s="14" t="n"/>
+      <c r="D9" s="14" t="n"/>
+      <c r="E9" s="15" t="n"/>
+      <c r="F9" s="20">
+        <f>IFERROR(E9/D9*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="17" t="n"/>
+      <c r="H9" s="14" t="n"/>
+      <c r="I9" s="15" t="n"/>
+      <c r="J9" s="20">
+        <f>IFERROR(I9/H9*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K9" s="21">
+        <f>E9+I9</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>August 2026</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="8">
-        <f>IFERROR(E9/D9*1000,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="B10" s="14" t="n"/>
+      <c r="C10" s="14" t="n"/>
+      <c r="D10" s="14" t="n"/>
+      <c r="E10" s="15" t="n"/>
+      <c r="F10" s="16">
+        <f>IFERROR(E10/D10*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="17" t="n"/>
+      <c r="H10" s="14" t="n"/>
+      <c r="I10" s="15" t="n"/>
+      <c r="J10" s="16">
+        <f>IFERROR(I10/H10*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K10" s="18">
+        <f>E10+I10</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>September 2026</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="7" t="n"/>
-      <c r="F10" s="10">
-        <f>IFERROR(E10/D10*1000,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="B11" s="14" t="n"/>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="14" t="n"/>
+      <c r="E11" s="15" t="n"/>
+      <c r="F11" s="20">
+        <f>IFERROR(E11/D11*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="17" t="n"/>
+      <c r="H11" s="14" t="n"/>
+      <c r="I11" s="15" t="n"/>
+      <c r="J11" s="20">
+        <f>IFERROR(I11/H11*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K11" s="21">
+        <f>E11+I11</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>October 2026</t>
         </is>
       </c>
-      <c r="B11" s="6" t="n"/>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="7" t="n"/>
-      <c r="F11" s="8">
-        <f>IFERROR(E11/D11*1000,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="B12" s="14" t="n"/>
+      <c r="C12" s="14" t="n"/>
+      <c r="D12" s="14" t="n"/>
+      <c r="E12" s="15" t="n"/>
+      <c r="F12" s="16">
+        <f>IFERROR(E12/D12*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G12" s="17" t="n"/>
+      <c r="H12" s="14" t="n"/>
+      <c r="I12" s="15" t="n"/>
+      <c r="J12" s="16">
+        <f>IFERROR(I12/H12*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K12" s="18">
+        <f>E12+I12</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>November 2026</t>
         </is>
       </c>
-      <c r="B12" s="6" t="n"/>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="7" t="n"/>
-      <c r="F12" s="10">
-        <f>IFERROR(E12/D12*1000,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="B13" s="14" t="n"/>
+      <c r="C13" s="14" t="n"/>
+      <c r="D13" s="14" t="n"/>
+      <c r="E13" s="15" t="n"/>
+      <c r="F13" s="20">
+        <f>IFERROR(E13/D13*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G13" s="17" t="n"/>
+      <c r="H13" s="14" t="n"/>
+      <c r="I13" s="15" t="n"/>
+      <c r="J13" s="20">
+        <f>IFERROR(I13/H13*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K13" s="21">
+        <f>E13+I13</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>December 2026</t>
         </is>
       </c>
-      <c r="B13" s="6" t="n"/>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="7" t="n"/>
-      <c r="F13" s="8">
-        <f>IFERROR(E13/D13*1000,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="B14" s="14" t="n"/>
+      <c r="C14" s="14" t="n"/>
+      <c r="D14" s="14" t="n"/>
+      <c r="E14" s="15" t="n"/>
+      <c r="F14" s="16">
+        <f>IFERROR(E14/D14*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G14" s="17" t="n"/>
+      <c r="H14" s="14" t="n"/>
+      <c r="I14" s="15" t="n"/>
+      <c r="J14" s="16">
+        <f>IFERROR(I14/H14*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K14" s="18">
+        <f>E14+I14</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>January 2027</t>
         </is>
       </c>
-      <c r="B14" s="6" t="n"/>
-      <c r="C14" s="6" t="n"/>
-      <c r="D14" s="6" t="n"/>
-      <c r="E14" s="7" t="n"/>
-      <c r="F14" s="10">
-        <f>IFERROR(E14/D14*1000,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="B15" s="14" t="n"/>
+      <c r="C15" s="14" t="n"/>
+      <c r="D15" s="14" t="n"/>
+      <c r="E15" s="15" t="n"/>
+      <c r="F15" s="20">
+        <f>IFERROR(E15/D15*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G15" s="17" t="n"/>
+      <c r="H15" s="14" t="n"/>
+      <c r="I15" s="15" t="n"/>
+      <c r="J15" s="20">
+        <f>IFERROR(I15/H15*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K15" s="21">
+        <f>E15+I15</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
         <is>
           <t>February 2027</t>
         </is>
       </c>
-      <c r="B15" s="6" t="n"/>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="7" t="n"/>
-      <c r="F15" s="8">
-        <f>IFERROR(E15/D15*1000,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="B16" s="14" t="n"/>
+      <c r="C16" s="14" t="n"/>
+      <c r="D16" s="14" t="n"/>
+      <c r="E16" s="15" t="n"/>
+      <c r="F16" s="16">
+        <f>IFERROR(E16/D16*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G16" s="17" t="n"/>
+      <c r="H16" s="14" t="n"/>
+      <c r="I16" s="15" t="n"/>
+      <c r="J16" s="16">
+        <f>IFERROR(I16/H16*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K16" s="18">
+        <f>E16+I16</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t>March 2027</t>
         </is>
       </c>
-      <c r="B16" s="6" t="n"/>
-      <c r="C16" s="6" t="n"/>
-      <c r="D16" s="6" t="n"/>
-      <c r="E16" s="7" t="n"/>
-      <c r="F16" s="10">
-        <f>IFERROR(E16/D16*1000,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" ht="10" customHeight="1"/>
-    <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="B17" s="14" t="n"/>
+      <c r="C17" s="14" t="n"/>
+      <c r="D17" s="14" t="n"/>
+      <c r="E17" s="15" t="n"/>
+      <c r="F17" s="20">
+        <f>IFERROR(E17/D17*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G17" s="17" t="n"/>
+      <c r="H17" s="14" t="n"/>
+      <c r="I17" s="15" t="n"/>
+      <c r="J17" s="20">
+        <f>IFERROR(I17/H17*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K17" s="21">
+        <f>E17+I17</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" ht="10" customHeight="1"/>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="22" t="inlineStr">
         <is>
           <t>SUMMARY</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="12" t="inlineStr">
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="23" t="inlineStr">
+        <is>
+          <t>Shorts</t>
+        </is>
+      </c>
+      <c r="B20" s="24" t="n"/>
+      <c r="C20" s="24" t="n"/>
+      <c r="D20" s="24" t="n"/>
+      <c r="E20" s="24" t="n"/>
+      <c r="F20" s="24" t="n"/>
+      <c r="G20" s="24" t="n"/>
+      <c r="H20" s="24" t="n"/>
+      <c r="I20" s="24" t="n"/>
+      <c r="J20" s="24" t="n"/>
+      <c r="K20" s="24" t="n"/>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="25" t="inlineStr">
+        <is>
+          <t>Total Shorts Published</t>
+        </is>
+      </c>
+      <c r="B21" s="26" t="n"/>
+      <c r="C21" s="26" t="n"/>
+      <c r="D21" s="26" t="n"/>
+      <c r="E21" s="26" t="n"/>
+      <c r="F21" s="26" t="n"/>
+      <c r="G21" s="26" t="n"/>
+      <c r="H21" s="26" t="n"/>
+      <c r="I21" s="26" t="n"/>
+      <c r="J21" s="26" t="n"/>
+      <c r="K21" s="27">
+        <f>SUM(B8:B17)</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="25" t="inlineStr">
+        <is>
+          <t>Total Views (Shorts)</t>
+        </is>
+      </c>
+      <c r="B22" s="26" t="n"/>
+      <c r="C22" s="26" t="n"/>
+      <c r="D22" s="26" t="n"/>
+      <c r="E22" s="26" t="n"/>
+      <c r="F22" s="26" t="n"/>
+      <c r="G22" s="26" t="n"/>
+      <c r="H22" s="26" t="n"/>
+      <c r="I22" s="26" t="n"/>
+      <c r="J22" s="26" t="n"/>
+      <c r="K22" s="27">
+        <f>SUM(C8:C17)</f>
+        <v>1100000</v>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="25" t="inlineStr">
+        <is>
+          <t>Total Engaged Views (Shorts)</t>
+        </is>
+      </c>
+      <c r="B23" s="26" t="n"/>
+      <c r="C23" s="26" t="n"/>
+      <c r="D23" s="26" t="n"/>
+      <c r="E23" s="26" t="n"/>
+      <c r="F23" s="26" t="n"/>
+      <c r="G23" s="26" t="n"/>
+      <c r="H23" s="26" t="n"/>
+      <c r="I23" s="26" t="n"/>
+      <c r="J23" s="26" t="n"/>
+      <c r="K23" s="27">
+        <f>SUM(D8:D17)</f>
+        <v>606700</v>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="25" t="inlineStr">
+        <is>
+          <t>Total Earnings (Shorts)</t>
+        </is>
+      </c>
+      <c r="B24" s="26" t="n"/>
+      <c r="C24" s="26" t="n"/>
+      <c r="D24" s="26" t="n"/>
+      <c r="E24" s="26" t="n"/>
+      <c r="F24" s="26" t="n"/>
+      <c r="G24" s="26" t="n"/>
+      <c r="H24" s="26" t="n"/>
+      <c r="I24" s="26" t="n"/>
+      <c r="J24" s="26" t="n"/>
+      <c r="K24" s="28">
+        <f>SUM(E8:E17)</f>
+        <v>146.81</v>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="25" t="inlineStr">
+        <is>
+          <t>Average RPM – Shorts (Earnings ÷ Engaged Views × 1000)</t>
+        </is>
+      </c>
+      <c r="B25" s="26" t="n"/>
+      <c r="C25" s="26" t="n"/>
+      <c r="D25" s="26" t="n"/>
+      <c r="E25" s="26" t="n"/>
+      <c r="F25" s="26" t="n"/>
+      <c r="G25" s="26" t="n"/>
+      <c r="H25" s="26" t="n"/>
+      <c r="I25" s="26" t="n"/>
+      <c r="J25" s="26" t="n"/>
+      <c r="K25" s="29">
+        <f>IFERROR(K24/K23*1000,0)</f>
+        <v>0.24198120982363605</v>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="30" t="inlineStr">
+        <is>
+          <t>Long-Form Videos</t>
+        </is>
+      </c>
+      <c r="B26" s="24" t="n"/>
+      <c r="C26" s="24" t="n"/>
+      <c r="D26" s="24" t="n"/>
+      <c r="E26" s="24" t="n"/>
+      <c r="F26" s="24" t="n"/>
+      <c r="G26" s="24" t="n"/>
+      <c r="H26" s="24" t="n"/>
+      <c r="I26" s="24" t="n"/>
+      <c r="J26" s="24" t="n"/>
+      <c r="K26" s="24" t="n"/>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="25" t="inlineStr">
         <is>
           <t>Total Videos Published</t>
         </is>
       </c>
-      <c r="B19" s="13" t="n"/>
-      <c r="C19" s="13" t="n"/>
-      <c r="D19" s="13" t="n"/>
-      <c r="E19" s="13" t="n"/>
-      <c r="F19" s="14">
-        <f>SUM(B7:B16)</f>
-        <v>18</v>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t>Total Views</t>
-        </is>
-      </c>
-      <c r="B20" s="13" t="n"/>
-      <c r="C20" s="13" t="n"/>
-      <c r="D20" s="13" t="n"/>
-      <c r="E20" s="13" t="n"/>
-      <c r="F20" s="14">
-        <f>SUM(C7:C16)</f>
-        <v>155000</v>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="12" t="inlineStr">
-        <is>
-          <t>Total Engaged Views</t>
-        </is>
-      </c>
-      <c r="B21" s="13" t="n"/>
-      <c r="C21" s="13" t="n"/>
-      <c r="D21" s="13" t="n"/>
-      <c r="E21" s="13" t="n"/>
-      <c r="F21" s="14">
-        <f>SUM(D7:D16)</f>
-        <v>130000</v>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="15" t="inlineStr">
-        <is>
-          <t>Total Earnings</t>
-        </is>
-      </c>
-      <c r="B22" s="16" t="n"/>
-      <c r="C22" s="16" t="n"/>
-      <c r="D22" s="16" t="n"/>
-      <c r="E22" s="16" t="n"/>
-      <c r="F22" s="17">
-        <f>SUM(E7:E16)</f>
-        <v>600</v>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="12" t="inlineStr">
-        <is>
-          <t>Average RPM (Total Earnings ÷ Total Engaged Views × 1000)</t>
-        </is>
-      </c>
-      <c r="B23" s="13" t="n"/>
-      <c r="C23" s="13" t="n"/>
-      <c r="D23" s="13" t="n"/>
-      <c r="E23" s="13" t="n"/>
-      <c r="F23" s="18">
-        <f>IFERROR(F22/F21*1000,0)</f>
-        <v>4.6153846153846154</v>
-      </c>
-    </row>
-    <row r="25" ht="42" customHeight="1">
-      <c r="A25" s="19" t="inlineStr">
-        <is>
-          <t>Note: "Engaged Views" are the monetized playbacks your revenue is actually paid on (YouTube Studio &gt; Analytics &gt; Revenue &gt; Playback-based CPM), which is why RPM and the Average RPM below are calculated against Engaged Views, not total Views. June and July 2026 are pre-filled with sample figures ($200 and $400 earnings) to show how the Summary adds up to $600 — replace them with your real numbers and fill in the remaining months as they happen.</t>
+      <c r="B27" s="26" t="n"/>
+      <c r="C27" s="26" t="n"/>
+      <c r="D27" s="26" t="n"/>
+      <c r="E27" s="26" t="n"/>
+      <c r="F27" s="26" t="n"/>
+      <c r="G27" s="26" t="n"/>
+      <c r="H27" s="26" t="n"/>
+      <c r="I27" s="26" t="n"/>
+      <c r="J27" s="26" t="n"/>
+      <c r="K27" s="27">
+        <f>SUM(G8:G17)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="25" t="inlineStr">
+        <is>
+          <t>Total Long Views</t>
+        </is>
+      </c>
+      <c r="B28" s="26" t="n"/>
+      <c r="C28" s="26" t="n"/>
+      <c r="D28" s="26" t="n"/>
+      <c r="E28" s="26" t="n"/>
+      <c r="F28" s="26" t="n"/>
+      <c r="G28" s="26" t="n"/>
+      <c r="H28" s="26" t="n"/>
+      <c r="I28" s="26" t="n"/>
+      <c r="J28" s="26" t="n"/>
+      <c r="K28" s="27">
+        <f>SUM(H8:H17)</f>
+        <v>31600</v>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="25" t="inlineStr">
+        <is>
+          <t>Total Earnings (Long-Form)</t>
+        </is>
+      </c>
+      <c r="B29" s="26" t="n"/>
+      <c r="C29" s="26" t="n"/>
+      <c r="D29" s="26" t="n"/>
+      <c r="E29" s="26" t="n"/>
+      <c r="F29" s="26" t="n"/>
+      <c r="G29" s="26" t="n"/>
+      <c r="H29" s="26" t="n"/>
+      <c r="I29" s="26" t="n"/>
+      <c r="J29" s="26" t="n"/>
+      <c r="K29" s="28">
+        <f>SUM(I8:I17)</f>
+        <v>59.84</v>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="25" t="inlineStr">
+        <is>
+          <t>Average RPM – Long-Form (Earnings ÷ Long Views × 1000)</t>
+        </is>
+      </c>
+      <c r="B30" s="26" t="n"/>
+      <c r="C30" s="26" t="n"/>
+      <c r="D30" s="26" t="n"/>
+      <c r="E30" s="26" t="n"/>
+      <c r="F30" s="26" t="n"/>
+      <c r="G30" s="26" t="n"/>
+      <c r="H30" s="26" t="n"/>
+      <c r="I30" s="26" t="n"/>
+      <c r="J30" s="26" t="n"/>
+      <c r="K30" s="29">
+        <f>IFERROR(K29/K28*1000,0)</f>
+        <v>1.8936708860759495</v>
+      </c>
+    </row>
+    <row r="32" ht="26" customHeight="1">
+      <c r="A32" s="31" t="inlineStr">
+        <is>
+          <t>TOTAL EARNINGS (Shorts + Long-Form, All Months)</t>
+        </is>
+      </c>
+      <c r="B32" s="32" t="n"/>
+      <c r="C32" s="32" t="n"/>
+      <c r="D32" s="32" t="n"/>
+      <c r="E32" s="32" t="n"/>
+      <c r="F32" s="32" t="n"/>
+      <c r="G32" s="32" t="n"/>
+      <c r="H32" s="32" t="n"/>
+      <c r="I32" s="32" t="n"/>
+      <c r="J32" s="32" t="n"/>
+      <c r="K32" s="33">
+        <f>SUM(K8:K17)</f>
+        <v>206.65</v>
+      </c>
+    </row>
+    <row r="34" ht="42" customHeight="1">
+      <c r="A34" s="34" t="inlineStr">
+        <is>
+          <t>Note: Shorts RPM is calculated on Engaged Views (the monetized playbacks Shorts revenue is paid on). Long-form RPM is calculated on total Long Views, since every long-form view is monetized. June 2026 is filled in with your real reported numbers; Total Earnings for that row is a formula (Earnings Shorts + Earnings Videos = $206.65) — enter your real figures for the remaining months as they happen.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="A21:E21"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="A23:E23"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="A25:F25"/>
+  <mergeCells count="21">
+    <mergeCell ref="A23:J23"/>
+    <mergeCell ref="A32:J32"/>
+    <mergeCell ref="A34:K34"/>
+    <mergeCell ref="A22:J22"/>
+    <mergeCell ref="A29:J29"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A28:J28"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A30:J30"/>
+    <mergeCell ref="A24:J24"/>
+    <mergeCell ref="A26:K26"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A25:J25"/>
+    <mergeCell ref="G6:J6"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="A20:K20"/>
+    <mergeCell ref="A27:J27"/>
+    <mergeCell ref="A21:J21"/>
+    <mergeCell ref="A19:K19"/>
+    <mergeCell ref="K6:K7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Extend earnings tracker back to channel start, mark pre-monetization months
Adds February–May 2026 to the top of the tracker (channel start date).
These months are shaded gray and labeled "(Pre-Monetization)": Views and
Published counts can still be logged, but Engaged Views, Earnings and RPM
are marked N/A since the channel wasn't monetized yet, and are excluded
from every earnings/RPM total via SUM's built-in text-skipping behavior.
Monetized tracking still begins June 2026 with the user's real numbers.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S454NQMsGhA62HZVzwmSTo
</commit_message>
<xml_diff>
--- a/YouTube_Earnings_Tracker.xlsx
+++ b/YouTube_Earnings_Tracker.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="166" formatCode="$#,##0.00"/>
     <numFmt numFmtId="167" formatCode="$0.00"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -63,12 +63,25 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001F2A44"/>
+      <i val="1"/>
+      <color rgb="009AA1AB"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <color rgb="0015417E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="009AA1AB"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F2A44"/>
       <sz val="10"/>
     </font>
     <font>
@@ -102,7 +115,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -126,12 +139,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4F6F8"/>
+        <fgColor rgb="00E7E9EC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EAF2FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4F6F8"/>
       </patternFill>
     </fill>
     <fill>
@@ -195,7 +213,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -235,55 +253,64 @@
     <xf numFmtId="3" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="12" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="14" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -654,10 +681,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
@@ -680,7 +707,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Reporting Period: June 2026 – March 2027</t>
+          <t>Reporting Period: February 2026 – March 2027</t>
         </is>
       </c>
     </row>
@@ -688,7 +715,7 @@
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Legend:  Pale blue cells = enter your monthly numbers   |   Blue text = your input   |   Navy text = auto-calculated formula   |   Shorts RPM uses Engaged Views, Long-form RPM uses total Long Views (you earn on every long-form view)</t>
+          <t>Legend:  Pale blue cells = enter your monthly numbers   |   Blue text = your input   |   Navy text = auto-calculated formula   |   Gray rows = pre-monetization (no earnings/RPM)   |   Shorts RPM uses Engaged Views, Long-form RPM uses total Long Views</t>
         </is>
       </c>
     </row>
@@ -774,549 +801,713 @@
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>June 2026</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>15</v>
-      </c>
-      <c r="C8" s="14" t="n">
-        <v>1100000</v>
-      </c>
-      <c r="D8" s="14" t="n">
-        <v>606700</v>
-      </c>
-      <c r="E8" s="15" t="n">
-        <v>146.81</v>
-      </c>
-      <c r="F8" s="16">
-        <f>IFERROR(E8/D8*1000,0)</f>
-        <v>0.24198120982363605</v>
-      </c>
-      <c r="G8" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" s="14" t="n">
-        <v>31600</v>
-      </c>
-      <c r="I8" s="15" t="n">
-        <v>59.84</v>
-      </c>
-      <c r="J8" s="16">
-        <f>IFERROR(I8/H8*1000,0)</f>
-        <v>1.8936708860759495</v>
-      </c>
-      <c r="K8" s="18">
-        <f>E8+I8</f>
-        <v>206.65</v>
+          <t>February 2026  (Pre-Monetization)</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="n"/>
+      <c r="C8" s="14" t="n"/>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G8" s="16" t="n"/>
+      <c r="H8" s="14" t="n"/>
+      <c r="I8" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J8" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K8" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>July 2026</t>
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>March 2026  (Pre-Monetization)</t>
         </is>
       </c>
       <c r="B9" s="14" t="n"/>
       <c r="C9" s="14" t="n"/>
-      <c r="D9" s="14" t="n"/>
-      <c r="E9" s="15" t="n"/>
-      <c r="F9" s="20">
-        <f>IFERROR(E9/D9*1000,0)</f>
-        <v>0</v>
-      </c>
-      <c r="G9" s="17" t="n"/>
+      <c r="D9" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F9" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="n"/>
       <c r="H9" s="14" t="n"/>
-      <c r="I9" s="15" t="n"/>
-      <c r="J9" s="20">
-        <f>IFERROR(I9/H9*1000,0)</f>
-        <v>0</v>
-      </c>
-      <c r="K9" s="21">
-        <f>E9+I9</f>
-        <v>0</v>
+      <c r="I9" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J9" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K9" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>August 2026</t>
+          <t>April 2026  (Pre-Monetization)</t>
         </is>
       </c>
       <c r="B10" s="14" t="n"/>
       <c r="C10" s="14" t="n"/>
-      <c r="D10" s="14" t="n"/>
-      <c r="E10" s="15" t="n"/>
-      <c r="F10" s="16">
-        <f>IFERROR(E10/D10*1000,0)</f>
-        <v>0</v>
-      </c>
-      <c r="G10" s="17" t="n"/>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F10" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G10" s="16" t="n"/>
       <c r="H10" s="14" t="n"/>
-      <c r="I10" s="15" t="n"/>
-      <c r="J10" s="16">
-        <f>IFERROR(I10/H10*1000,0)</f>
-        <v>0</v>
-      </c>
-      <c r="K10" s="18">
-        <f>E10+I10</f>
-        <v>0</v>
+      <c r="I10" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J10" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K10" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>September 2026</t>
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>May 2026  (Pre-Monetization)</t>
         </is>
       </c>
       <c r="B11" s="14" t="n"/>
       <c r="C11" s="14" t="n"/>
-      <c r="D11" s="14" t="n"/>
-      <c r="E11" s="15" t="n"/>
-      <c r="F11" s="20">
-        <f>IFERROR(E11/D11*1000,0)</f>
-        <v>0</v>
-      </c>
-      <c r="G11" s="17" t="n"/>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F11" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="n"/>
       <c r="H11" s="14" t="n"/>
-      <c r="I11" s="15" t="n"/>
-      <c r="J11" s="20">
-        <f>IFERROR(I11/H11*1000,0)</f>
-        <v>0</v>
-      </c>
-      <c r="K11" s="21">
-        <f>E11+I11</f>
-        <v>0</v>
+      <c r="I11" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J11" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K11" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>October 2026</t>
-        </is>
-      </c>
-      <c r="B12" s="14" t="n"/>
-      <c r="C12" s="14" t="n"/>
-      <c r="D12" s="14" t="n"/>
-      <c r="E12" s="15" t="n"/>
-      <c r="F12" s="16">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>June 2026</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="C12" s="14" t="n">
+        <v>1100000</v>
+      </c>
+      <c r="D12" s="14" t="n">
+        <v>606700</v>
+      </c>
+      <c r="E12" s="19" t="n">
+        <v>146.81</v>
+      </c>
+      <c r="F12" s="20">
         <f>IFERROR(E12/D12*1000,0)</f>
-        <v>0</v>
-      </c>
-      <c r="G12" s="17" t="n"/>
-      <c r="H12" s="14" t="n"/>
-      <c r="I12" s="15" t="n"/>
-      <c r="J12" s="16">
+        <v>0.24198120982363605</v>
+      </c>
+      <c r="G12" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="14" t="n">
+        <v>31600</v>
+      </c>
+      <c r="I12" s="19" t="n">
+        <v>59.84</v>
+      </c>
+      <c r="J12" s="20">
         <f>IFERROR(I12/H12*1000,0)</f>
-        <v>0</v>
-      </c>
-      <c r="K12" s="18">
+        <v>1.8936708860759495</v>
+      </c>
+      <c r="K12" s="21">
         <f>E12+I12</f>
-        <v>0</v>
+        <v>206.65</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>November 2026</t>
+      <c r="A13" s="22" t="inlineStr">
+        <is>
+          <t>July 2026</t>
         </is>
       </c>
       <c r="B13" s="14" t="n"/>
       <c r="C13" s="14" t="n"/>
       <c r="D13" s="14" t="n"/>
-      <c r="E13" s="15" t="n"/>
-      <c r="F13" s="20">
+      <c r="E13" s="19" t="n"/>
+      <c r="F13" s="23">
         <f>IFERROR(E13/D13*1000,0)</f>
         <v>0</v>
       </c>
-      <c r="G13" s="17" t="n"/>
+      <c r="G13" s="16" t="n"/>
       <c r="H13" s="14" t="n"/>
-      <c r="I13" s="15" t="n"/>
-      <c r="J13" s="20">
+      <c r="I13" s="19" t="n"/>
+      <c r="J13" s="23">
         <f>IFERROR(I13/H13*1000,0)</f>
         <v>0</v>
       </c>
-      <c r="K13" s="21">
+      <c r="K13" s="24">
         <f>E13+I13</f>
         <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
-        <is>
-          <t>December 2026</t>
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>August 2026</t>
         </is>
       </c>
       <c r="B14" s="14" t="n"/>
       <c r="C14" s="14" t="n"/>
       <c r="D14" s="14" t="n"/>
-      <c r="E14" s="15" t="n"/>
-      <c r="F14" s="16">
+      <c r="E14" s="19" t="n"/>
+      <c r="F14" s="20">
         <f>IFERROR(E14/D14*1000,0)</f>
         <v>0</v>
       </c>
-      <c r="G14" s="17" t="n"/>
+      <c r="G14" s="16" t="n"/>
       <c r="H14" s="14" t="n"/>
-      <c r="I14" s="15" t="n"/>
-      <c r="J14" s="16">
+      <c r="I14" s="19" t="n"/>
+      <c r="J14" s="20">
         <f>IFERROR(I14/H14*1000,0)</f>
         <v>0</v>
       </c>
-      <c r="K14" s="18">
+      <c r="K14" s="21">
         <f>E14+I14</f>
         <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
-        <is>
-          <t>January 2027</t>
+      <c r="A15" s="22" t="inlineStr">
+        <is>
+          <t>September 2026</t>
         </is>
       </c>
       <c r="B15" s="14" t="n"/>
       <c r="C15" s="14" t="n"/>
       <c r="D15" s="14" t="n"/>
-      <c r="E15" s="15" t="n"/>
-      <c r="F15" s="20">
+      <c r="E15" s="19" t="n"/>
+      <c r="F15" s="23">
         <f>IFERROR(E15/D15*1000,0)</f>
         <v>0</v>
       </c>
-      <c r="G15" s="17" t="n"/>
+      <c r="G15" s="16" t="n"/>
       <c r="H15" s="14" t="n"/>
-      <c r="I15" s="15" t="n"/>
-      <c r="J15" s="20">
+      <c r="I15" s="19" t="n"/>
+      <c r="J15" s="23">
         <f>IFERROR(I15/H15*1000,0)</f>
         <v>0</v>
       </c>
-      <c r="K15" s="21">
+      <c r="K15" s="24">
         <f>E15+I15</f>
         <v>0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="inlineStr">
-        <is>
-          <t>February 2027</t>
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>October 2026</t>
         </is>
       </c>
       <c r="B16" s="14" t="n"/>
       <c r="C16" s="14" t="n"/>
       <c r="D16" s="14" t="n"/>
-      <c r="E16" s="15" t="n"/>
-      <c r="F16" s="16">
+      <c r="E16" s="19" t="n"/>
+      <c r="F16" s="20">
         <f>IFERROR(E16/D16*1000,0)</f>
         <v>0</v>
       </c>
-      <c r="G16" s="17" t="n"/>
+      <c r="G16" s="16" t="n"/>
       <c r="H16" s="14" t="n"/>
-      <c r="I16" s="15" t="n"/>
-      <c r="J16" s="16">
+      <c r="I16" s="19" t="n"/>
+      <c r="J16" s="20">
         <f>IFERROR(I16/H16*1000,0)</f>
         <v>0</v>
       </c>
-      <c r="K16" s="18">
+      <c r="K16" s="21">
         <f>E16+I16</f>
         <v>0</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
-        <is>
-          <t>March 2027</t>
+      <c r="A17" s="22" t="inlineStr">
+        <is>
+          <t>November 2026</t>
         </is>
       </c>
       <c r="B17" s="14" t="n"/>
       <c r="C17" s="14" t="n"/>
       <c r="D17" s="14" t="n"/>
-      <c r="E17" s="15" t="n"/>
-      <c r="F17" s="20">
+      <c r="E17" s="19" t="n"/>
+      <c r="F17" s="23">
         <f>IFERROR(E17/D17*1000,0)</f>
         <v>0</v>
       </c>
-      <c r="G17" s="17" t="n"/>
+      <c r="G17" s="16" t="n"/>
       <c r="H17" s="14" t="n"/>
-      <c r="I17" s="15" t="n"/>
-      <c r="J17" s="20">
+      <c r="I17" s="19" t="n"/>
+      <c r="J17" s="23">
         <f>IFERROR(I17/H17*1000,0)</f>
         <v>0</v>
       </c>
-      <c r="K17" s="21">
+      <c r="K17" s="24">
         <f>E17+I17</f>
         <v>0</v>
       </c>
     </row>
-    <row r="18" ht="10" customHeight="1"/>
-    <row r="19" ht="24" customHeight="1">
+    <row r="18">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>December 2026</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="n"/>
+      <c r="C18" s="14" t="n"/>
+      <c r="D18" s="14" t="n"/>
+      <c r="E18" s="19" t="n"/>
+      <c r="F18" s="20">
+        <f>IFERROR(E18/D18*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G18" s="16" t="n"/>
+      <c r="H18" s="14" t="n"/>
+      <c r="I18" s="19" t="n"/>
+      <c r="J18" s="20">
+        <f>IFERROR(I18/H18*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K18" s="21">
+        <f>E18+I18</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
       <c r="A19" s="22" t="inlineStr">
         <is>
+          <t>January 2027</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="n"/>
+      <c r="C19" s="14" t="n"/>
+      <c r="D19" s="14" t="n"/>
+      <c r="E19" s="19" t="n"/>
+      <c r="F19" s="23">
+        <f>IFERROR(E19/D19*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G19" s="16" t="n"/>
+      <c r="H19" s="14" t="n"/>
+      <c r="I19" s="19" t="n"/>
+      <c r="J19" s="23">
+        <f>IFERROR(I19/H19*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K19" s="24">
+        <f>E19+I19</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>February 2027</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="n"/>
+      <c r="C20" s="14" t="n"/>
+      <c r="D20" s="14" t="n"/>
+      <c r="E20" s="19" t="n"/>
+      <c r="F20" s="20">
+        <f>IFERROR(E20/D20*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G20" s="16" t="n"/>
+      <c r="H20" s="14" t="n"/>
+      <c r="I20" s="19" t="n"/>
+      <c r="J20" s="20">
+        <f>IFERROR(I20/H20*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K20" s="21">
+        <f>E20+I20</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="22" t="inlineStr">
+        <is>
+          <t>March 2027</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="n"/>
+      <c r="C21" s="14" t="n"/>
+      <c r="D21" s="14" t="n"/>
+      <c r="E21" s="19" t="n"/>
+      <c r="F21" s="23">
+        <f>IFERROR(E21/D21*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G21" s="16" t="n"/>
+      <c r="H21" s="14" t="n"/>
+      <c r="I21" s="19" t="n"/>
+      <c r="J21" s="23">
+        <f>IFERROR(I21/H21*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K21" s="24">
+        <f>E21+I21</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" ht="10" customHeight="1"/>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="25" t="inlineStr">
+        <is>
           <t>SUMMARY</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="23" t="inlineStr">
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="26" t="inlineStr">
         <is>
           <t>Shorts</t>
         </is>
       </c>
-      <c r="B20" s="24" t="n"/>
-      <c r="C20" s="24" t="n"/>
-      <c r="D20" s="24" t="n"/>
-      <c r="E20" s="24" t="n"/>
-      <c r="F20" s="24" t="n"/>
-      <c r="G20" s="24" t="n"/>
-      <c r="H20" s="24" t="n"/>
-      <c r="I20" s="24" t="n"/>
-      <c r="J20" s="24" t="n"/>
-      <c r="K20" s="24" t="n"/>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="25" t="inlineStr">
+      <c r="B24" s="27" t="n"/>
+      <c r="C24" s="27" t="n"/>
+      <c r="D24" s="27" t="n"/>
+      <c r="E24" s="27" t="n"/>
+      <c r="F24" s="27" t="n"/>
+      <c r="G24" s="27" t="n"/>
+      <c r="H24" s="27" t="n"/>
+      <c r="I24" s="27" t="n"/>
+      <c r="J24" s="27" t="n"/>
+      <c r="K24" s="27" t="n"/>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="28" t="inlineStr">
         <is>
           <t>Total Shorts Published</t>
         </is>
       </c>
-      <c r="B21" s="26" t="n"/>
-      <c r="C21" s="26" t="n"/>
-      <c r="D21" s="26" t="n"/>
-      <c r="E21" s="26" t="n"/>
-      <c r="F21" s="26" t="n"/>
-      <c r="G21" s="26" t="n"/>
-      <c r="H21" s="26" t="n"/>
-      <c r="I21" s="26" t="n"/>
-      <c r="J21" s="26" t="n"/>
-      <c r="K21" s="27">
-        <f>SUM(B8:B17)</f>
+      <c r="B25" s="29" t="n"/>
+      <c r="C25" s="29" t="n"/>
+      <c r="D25" s="29" t="n"/>
+      <c r="E25" s="29" t="n"/>
+      <c r="F25" s="29" t="n"/>
+      <c r="G25" s="29" t="n"/>
+      <c r="H25" s="29" t="n"/>
+      <c r="I25" s="29" t="n"/>
+      <c r="J25" s="29" t="n"/>
+      <c r="K25" s="30">
+        <f>SUM(B8:B21)</f>
         <v>15</v>
       </c>
     </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="25" t="inlineStr">
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="28" t="inlineStr">
         <is>
           <t>Total Views (Shorts)</t>
         </is>
       </c>
-      <c r="B22" s="26" t="n"/>
-      <c r="C22" s="26" t="n"/>
-      <c r="D22" s="26" t="n"/>
-      <c r="E22" s="26" t="n"/>
-      <c r="F22" s="26" t="n"/>
-      <c r="G22" s="26" t="n"/>
-      <c r="H22" s="26" t="n"/>
-      <c r="I22" s="26" t="n"/>
-      <c r="J22" s="26" t="n"/>
-      <c r="K22" s="27">
-        <f>SUM(C8:C17)</f>
+      <c r="B26" s="29" t="n"/>
+      <c r="C26" s="29" t="n"/>
+      <c r="D26" s="29" t="n"/>
+      <c r="E26" s="29" t="n"/>
+      <c r="F26" s="29" t="n"/>
+      <c r="G26" s="29" t="n"/>
+      <c r="H26" s="29" t="n"/>
+      <c r="I26" s="29" t="n"/>
+      <c r="J26" s="29" t="n"/>
+      <c r="K26" s="30">
+        <f>SUM(C8:C21)</f>
         <v>1100000</v>
       </c>
     </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="25" t="inlineStr">
-        <is>
-          <t>Total Engaged Views (Shorts)</t>
-        </is>
-      </c>
-      <c r="B23" s="26" t="n"/>
-      <c r="C23" s="26" t="n"/>
-      <c r="D23" s="26" t="n"/>
-      <c r="E23" s="26" t="n"/>
-      <c r="F23" s="26" t="n"/>
-      <c r="G23" s="26" t="n"/>
-      <c r="H23" s="26" t="n"/>
-      <c r="I23" s="26" t="n"/>
-      <c r="J23" s="26" t="n"/>
-      <c r="K23" s="27">
-        <f>SUM(D8:D17)</f>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="28" t="inlineStr">
+        <is>
+          <t>Total Engaged Views (Shorts, monetized months only)</t>
+        </is>
+      </c>
+      <c r="B27" s="29" t="n"/>
+      <c r="C27" s="29" t="n"/>
+      <c r="D27" s="29" t="n"/>
+      <c r="E27" s="29" t="n"/>
+      <c r="F27" s="29" t="n"/>
+      <c r="G27" s="29" t="n"/>
+      <c r="H27" s="29" t="n"/>
+      <c r="I27" s="29" t="n"/>
+      <c r="J27" s="29" t="n"/>
+      <c r="K27" s="30">
+        <f>SUM(D8:D21)</f>
         <v>606700</v>
       </c>
     </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="25" t="inlineStr">
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="28" t="inlineStr">
         <is>
           <t>Total Earnings (Shorts)</t>
         </is>
       </c>
-      <c r="B24" s="26" t="n"/>
-      <c r="C24" s="26" t="n"/>
-      <c r="D24" s="26" t="n"/>
-      <c r="E24" s="26" t="n"/>
-      <c r="F24" s="26" t="n"/>
-      <c r="G24" s="26" t="n"/>
-      <c r="H24" s="26" t="n"/>
-      <c r="I24" s="26" t="n"/>
-      <c r="J24" s="26" t="n"/>
-      <c r="K24" s="28">
-        <f>SUM(E8:E17)</f>
+      <c r="B28" s="29" t="n"/>
+      <c r="C28" s="29" t="n"/>
+      <c r="D28" s="29" t="n"/>
+      <c r="E28" s="29" t="n"/>
+      <c r="F28" s="29" t="n"/>
+      <c r="G28" s="29" t="n"/>
+      <c r="H28" s="29" t="n"/>
+      <c r="I28" s="29" t="n"/>
+      <c r="J28" s="29" t="n"/>
+      <c r="K28" s="31">
+        <f>SUM(E8:E21)</f>
         <v>146.81</v>
       </c>
     </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="25" t="inlineStr">
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="28" t="inlineStr">
         <is>
           <t>Average RPM – Shorts (Earnings ÷ Engaged Views × 1000)</t>
         </is>
       </c>
-      <c r="B25" s="26" t="n"/>
-      <c r="C25" s="26" t="n"/>
-      <c r="D25" s="26" t="n"/>
-      <c r="E25" s="26" t="n"/>
-      <c r="F25" s="26" t="n"/>
-      <c r="G25" s="26" t="n"/>
-      <c r="H25" s="26" t="n"/>
-      <c r="I25" s="26" t="n"/>
-      <c r="J25" s="26" t="n"/>
-      <c r="K25" s="29">
-        <f>IFERROR(K24/K23*1000,0)</f>
+      <c r="B29" s="29" t="n"/>
+      <c r="C29" s="29" t="n"/>
+      <c r="D29" s="29" t="n"/>
+      <c r="E29" s="29" t="n"/>
+      <c r="F29" s="29" t="n"/>
+      <c r="G29" s="29" t="n"/>
+      <c r="H29" s="29" t="n"/>
+      <c r="I29" s="29" t="n"/>
+      <c r="J29" s="29" t="n"/>
+      <c r="K29" s="32">
+        <f>IFERROR(K28/K27*1000,0)</f>
         <v>0.24198120982363605</v>
       </c>
     </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="30" t="inlineStr">
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="33" t="inlineStr">
         <is>
           <t>Long-Form Videos</t>
         </is>
       </c>
-      <c r="B26" s="24" t="n"/>
-      <c r="C26" s="24" t="n"/>
-      <c r="D26" s="24" t="n"/>
-      <c r="E26" s="24" t="n"/>
-      <c r="F26" s="24" t="n"/>
-      <c r="G26" s="24" t="n"/>
-      <c r="H26" s="24" t="n"/>
-      <c r="I26" s="24" t="n"/>
-      <c r="J26" s="24" t="n"/>
-      <c r="K26" s="24" t="n"/>
-    </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="25" t="inlineStr">
+      <c r="B30" s="27" t="n"/>
+      <c r="C30" s="27" t="n"/>
+      <c r="D30" s="27" t="n"/>
+      <c r="E30" s="27" t="n"/>
+      <c r="F30" s="27" t="n"/>
+      <c r="G30" s="27" t="n"/>
+      <c r="H30" s="27" t="n"/>
+      <c r="I30" s="27" t="n"/>
+      <c r="J30" s="27" t="n"/>
+      <c r="K30" s="27" t="n"/>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="28" t="inlineStr">
         <is>
           <t>Total Videos Published</t>
         </is>
       </c>
-      <c r="B27" s="26" t="n"/>
-      <c r="C27" s="26" t="n"/>
-      <c r="D27" s="26" t="n"/>
-      <c r="E27" s="26" t="n"/>
-      <c r="F27" s="26" t="n"/>
-      <c r="G27" s="26" t="n"/>
-      <c r="H27" s="26" t="n"/>
-      <c r="I27" s="26" t="n"/>
-      <c r="J27" s="26" t="n"/>
-      <c r="K27" s="27">
-        <f>SUM(G8:G17)</f>
+      <c r="B31" s="29" t="n"/>
+      <c r="C31" s="29" t="n"/>
+      <c r="D31" s="29" t="n"/>
+      <c r="E31" s="29" t="n"/>
+      <c r="F31" s="29" t="n"/>
+      <c r="G31" s="29" t="n"/>
+      <c r="H31" s="29" t="n"/>
+      <c r="I31" s="29" t="n"/>
+      <c r="J31" s="29" t="n"/>
+      <c r="K31" s="30">
+        <f>SUM(G8:G21)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="25" t="inlineStr">
-        <is>
-          <t>Total Long Views</t>
-        </is>
-      </c>
-      <c r="B28" s="26" t="n"/>
-      <c r="C28" s="26" t="n"/>
-      <c r="D28" s="26" t="n"/>
-      <c r="E28" s="26" t="n"/>
-      <c r="F28" s="26" t="n"/>
-      <c r="G28" s="26" t="n"/>
-      <c r="H28" s="26" t="n"/>
-      <c r="I28" s="26" t="n"/>
-      <c r="J28" s="26" t="n"/>
-      <c r="K28" s="27">
-        <f>SUM(H8:H17)</f>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="28" t="inlineStr">
+        <is>
+          <t>Total Long Views (monetized months only)</t>
+        </is>
+      </c>
+      <c r="B32" s="29" t="n"/>
+      <c r="C32" s="29" t="n"/>
+      <c r="D32" s="29" t="n"/>
+      <c r="E32" s="29" t="n"/>
+      <c r="F32" s="29" t="n"/>
+      <c r="G32" s="29" t="n"/>
+      <c r="H32" s="29" t="n"/>
+      <c r="I32" s="29" t="n"/>
+      <c r="J32" s="29" t="n"/>
+      <c r="K32" s="30">
+        <f>SUM(H8:H21)</f>
         <v>31600</v>
       </c>
     </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="25" t="inlineStr">
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="28" t="inlineStr">
         <is>
           <t>Total Earnings (Long-Form)</t>
         </is>
       </c>
-      <c r="B29" s="26" t="n"/>
-      <c r="C29" s="26" t="n"/>
-      <c r="D29" s="26" t="n"/>
-      <c r="E29" s="26" t="n"/>
-      <c r="F29" s="26" t="n"/>
-      <c r="G29" s="26" t="n"/>
-      <c r="H29" s="26" t="n"/>
-      <c r="I29" s="26" t="n"/>
-      <c r="J29" s="26" t="n"/>
-      <c r="K29" s="28">
-        <f>SUM(I8:I17)</f>
+      <c r="B33" s="29" t="n"/>
+      <c r="C33" s="29" t="n"/>
+      <c r="D33" s="29" t="n"/>
+      <c r="E33" s="29" t="n"/>
+      <c r="F33" s="29" t="n"/>
+      <c r="G33" s="29" t="n"/>
+      <c r="H33" s="29" t="n"/>
+      <c r="I33" s="29" t="n"/>
+      <c r="J33" s="29" t="n"/>
+      <c r="K33" s="31">
+        <f>SUM(I8:I21)</f>
         <v>59.84</v>
       </c>
     </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="25" t="inlineStr">
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="28" t="inlineStr">
         <is>
           <t>Average RPM – Long-Form (Earnings ÷ Long Views × 1000)</t>
         </is>
       </c>
-      <c r="B30" s="26" t="n"/>
-      <c r="C30" s="26" t="n"/>
-      <c r="D30" s="26" t="n"/>
-      <c r="E30" s="26" t="n"/>
-      <c r="F30" s="26" t="n"/>
-      <c r="G30" s="26" t="n"/>
-      <c r="H30" s="26" t="n"/>
-      <c r="I30" s="26" t="n"/>
-      <c r="J30" s="26" t="n"/>
-      <c r="K30" s="29">
-        <f>IFERROR(K29/K28*1000,0)</f>
+      <c r="B34" s="29" t="n"/>
+      <c r="C34" s="29" t="n"/>
+      <c r="D34" s="29" t="n"/>
+      <c r="E34" s="29" t="n"/>
+      <c r="F34" s="29" t="n"/>
+      <c r="G34" s="29" t="n"/>
+      <c r="H34" s="29" t="n"/>
+      <c r="I34" s="29" t="n"/>
+      <c r="J34" s="29" t="n"/>
+      <c r="K34" s="32">
+        <f>IFERROR(K33/K32*1000,0)</f>
         <v>1.8936708860759495</v>
       </c>
     </row>
-    <row r="32" ht="26" customHeight="1">
-      <c r="A32" s="31" t="inlineStr">
+    <row r="36" ht="26" customHeight="1">
+      <c r="A36" s="34" t="inlineStr">
         <is>
           <t>TOTAL EARNINGS (Shorts + Long-Form, All Months)</t>
         </is>
       </c>
-      <c r="B32" s="32" t="n"/>
-      <c r="C32" s="32" t="n"/>
-      <c r="D32" s="32" t="n"/>
-      <c r="E32" s="32" t="n"/>
-      <c r="F32" s="32" t="n"/>
-      <c r="G32" s="32" t="n"/>
-      <c r="H32" s="32" t="n"/>
-      <c r="I32" s="32" t="n"/>
-      <c r="J32" s="32" t="n"/>
-      <c r="K32" s="33">
-        <f>SUM(K8:K17)</f>
+      <c r="B36" s="35" t="n"/>
+      <c r="C36" s="35" t="n"/>
+      <c r="D36" s="35" t="n"/>
+      <c r="E36" s="35" t="n"/>
+      <c r="F36" s="35" t="n"/>
+      <c r="G36" s="35" t="n"/>
+      <c r="H36" s="35" t="n"/>
+      <c r="I36" s="35" t="n"/>
+      <c r="J36" s="35" t="n"/>
+      <c r="K36" s="36">
+        <f>SUM(K8:K21)</f>
         <v>206.65</v>
       </c>
     </row>
-    <row r="34" ht="42" customHeight="1">
-      <c r="A34" s="34" t="inlineStr">
-        <is>
-          <t>Note: Shorts RPM is calculated on Engaged Views (the monetized playbacks Shorts revenue is paid on). Long-form RPM is calculated on total Long Views, since every long-form view is monetized. June 2026 is filled in with your real reported numbers; Total Earnings for that row is a formula (Earnings Shorts + Earnings Videos = $206.65) — enter your real figures for the remaining months as they happen.</t>
+    <row r="38" ht="56" customHeight="1">
+      <c r="A38" s="37" t="inlineStr">
+        <is>
+          <t>Note: February–May 2026 are shaded gray because the channel wasn't monetized yet — Videos/Shorts Published and Views can still be logged, but Engaged Views, Earnings and RPM are marked N/A and excluded from every earnings/RPM total below. Monetized tracking begins June 2026, filled in with your real reported numbers (Shorts $146.81 + Long-Form $59.84 = $206.65). Shorts RPM is calculated on Engaged Views; Long-Form RPM is calculated on total Long Views, since every long-form view is monetized. Enter your real figures for the remaining months as they happen.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="A23:J23"/>
     <mergeCell ref="A32:J32"/>
-    <mergeCell ref="A34:K34"/>
-    <mergeCell ref="A22:J22"/>
+    <mergeCell ref="A30:K30"/>
+    <mergeCell ref="A24:K24"/>
     <mergeCell ref="A29:J29"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A28:J28"/>
     <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A30:J30"/>
-    <mergeCell ref="A24:J24"/>
-    <mergeCell ref="A26:K26"/>
+    <mergeCell ref="A31:J31"/>
+    <mergeCell ref="A34:J34"/>
+    <mergeCell ref="A36:J36"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A25:J25"/>
+    <mergeCell ref="A23:K23"/>
     <mergeCell ref="G6:J6"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="B6:F6"/>
-    <mergeCell ref="A20:K20"/>
     <mergeCell ref="A27:J27"/>
-    <mergeCell ref="A21:J21"/>
-    <mergeCell ref="A19:K19"/>
+    <mergeCell ref="A38:K38"/>
     <mergeCell ref="K6:K7"/>
+    <mergeCell ref="A26:J26"/>
+    <mergeCell ref="A33:J33"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Exclude pre-monetization Long Views from the RPM average
Total Long Views (and the paired Shorts Engaged Views / Earnings totals)
now sum only the monetized months (June 2026 onward) instead of the full
Feb 2026 - Mar 2027 range. Previously, any Long Views logged during the
pre-monetization Feb-May 2026 window would have diluted the Long-Form
RPM average, since that column stays fillable even before monetization
starts (unlike Engaged Views/Earnings, which are marked N/A).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S454NQMsGhA62HZVzwmSTo
</commit_message>
<xml_diff>
--- a/YouTube_Earnings_Tracker.xlsx
+++ b/YouTube_Earnings_Tracker.xlsx
@@ -1317,7 +1317,7 @@
       <c r="I27" s="29" t="n"/>
       <c r="J27" s="29" t="n"/>
       <c r="K27" s="30">
-        <f>SUM(D8:D21)</f>
+        <f>SUM(D12:D21)</f>
         <v>606700</v>
       </c>
     </row>
@@ -1337,7 +1337,7 @@
       <c r="I28" s="29" t="n"/>
       <c r="J28" s="29" t="n"/>
       <c r="K28" s="31">
-        <f>SUM(E8:E21)</f>
+        <f>SUM(E12:E21)</f>
         <v>146.81</v>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       <c r="I32" s="29" t="n"/>
       <c r="J32" s="29" t="n"/>
       <c r="K32" s="30">
-        <f>SUM(H8:H21)</f>
+        <f>SUM(H12:H21)</f>
         <v>31600</v>
       </c>
     </row>
@@ -1434,7 +1434,7 @@
       <c r="I33" s="29" t="n"/>
       <c r="J33" s="29" t="n"/>
       <c r="K33" s="31">
-        <f>SUM(I8:I21)</f>
+        <f>SUM(I12:I21)</f>
         <v>59.84</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Feb-Apr pre-monetization data, move monetization start to May 2026
Fills in the user's real Feb, March, and April 2026 stats (Shorts
Published, Views, Videos Published, Long Views) as pre-monetization
rows, and corrects the monetization start date from June to May 2026
per the user's clarification. May 2026 is now a fully monetized row
with real Engaged Views, Earnings, and RPM (Shorts $10.85 + Long-Form
$6.42 = $17.27), pushing the running grand total to $223.92.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S454NQMsGhA62HZVzwmSTo
</commit_message>
<xml_diff>
--- a/YouTube_Earnings_Tracker.xlsx
+++ b/YouTube_Earnings_Tracker.xlsx
@@ -149,12 +149,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4F6F8"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="00F4F6F8"/>
       </patternFill>
     </fill>
     <fill>
@@ -294,13 +294,13 @@
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="9" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -804,8 +804,12 @@
           <t>February 2026  (Pre-Monetization)</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n"/>
-      <c r="C8" s="14" t="n"/>
+      <c r="B8" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>3400000</v>
+      </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -821,8 +825,12 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="G8" s="16" t="n"/>
-      <c r="H8" s="14" t="n"/>
+      <c r="G8" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="14" t="n">
+        <v>2200</v>
+      </c>
       <c r="I8" s="15" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -845,8 +853,12 @@
           <t>March 2026  (Pre-Monetization)</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n"/>
-      <c r="C9" s="14" t="n"/>
+      <c r="B9" s="14" t="n">
+        <v>26</v>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>5700000</v>
+      </c>
       <c r="D9" s="15" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -862,8 +874,12 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="G9" s="16" t="n"/>
-      <c r="H9" s="14" t="n"/>
+      <c r="G9" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="14" t="n">
+        <v>40200</v>
+      </c>
       <c r="I9" s="15" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -886,8 +902,12 @@
           <t>April 2026  (Pre-Monetization)</t>
         </is>
       </c>
-      <c r="B10" s="14" t="n"/>
-      <c r="C10" s="14" t="n"/>
+      <c r="B10" s="14" t="n">
+        <v>14</v>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>3100000</v>
+      </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -903,8 +923,12 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="G10" s="16" t="n"/>
-      <c r="H10" s="14" t="n"/>
+      <c r="G10" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" s="14" t="n">
+        <v>35200</v>
+      </c>
       <c r="I10" s="15" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -922,48 +946,47 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
-        <is>
-          <t>May 2026  (Pre-Monetization)</t>
-        </is>
-      </c>
-      <c r="B11" s="14" t="n"/>
-      <c r="C11" s="14" t="n"/>
-      <c r="D11" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E11" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F11" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G11" s="16" t="n"/>
-      <c r="H11" s="14" t="n"/>
-      <c r="I11" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="J11" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K11" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="C11" s="14" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D11" s="14" t="n">
+        <v>43300</v>
+      </c>
+      <c r="E11" s="19" t="n">
+        <v>10.85</v>
+      </c>
+      <c r="F11" s="20">
+        <f>IFERROR(E11/D11*1000,0)</f>
+        <v>0.2505773672055427</v>
+      </c>
+      <c r="G11" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" s="14" t="n">
+        <v>6400</v>
+      </c>
+      <c r="I11" s="19" t="n">
+        <v>6.42</v>
+      </c>
+      <c r="J11" s="20">
+        <f>IFERROR(I11/H11*1000,0)</f>
+        <v>1.0031249999999998</v>
+      </c>
+      <c r="K11" s="21">
+        <f>E11+I11</f>
+        <v>17.27</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>June 2026</t>
         </is>
@@ -980,7 +1003,7 @@
       <c r="E12" s="19" t="n">
         <v>146.81</v>
       </c>
-      <c r="F12" s="20">
+      <c r="F12" s="23">
         <f>IFERROR(E12/D12*1000,0)</f>
         <v>0.24198120982363605</v>
       </c>
@@ -993,17 +1016,17 @@
       <c r="I12" s="19" t="n">
         <v>59.84</v>
       </c>
-      <c r="J12" s="20">
+      <c r="J12" s="23">
         <f>IFERROR(I12/H12*1000,0)</f>
         <v>1.8936708860759495</v>
       </c>
-      <c r="K12" s="21">
+      <c r="K12" s="24">
         <f>E12+I12</f>
         <v>206.65</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="22" t="inlineStr">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>July 2026</t>
         </is>
@@ -1012,24 +1035,24 @@
       <c r="C13" s="14" t="n"/>
       <c r="D13" s="14" t="n"/>
       <c r="E13" s="19" t="n"/>
-      <c r="F13" s="23">
+      <c r="F13" s="20">
         <f>IFERROR(E13/D13*1000,0)</f>
         <v>0</v>
       </c>
       <c r="G13" s="16" t="n"/>
       <c r="H13" s="14" t="n"/>
       <c r="I13" s="19" t="n"/>
-      <c r="J13" s="23">
+      <c r="J13" s="20">
         <f>IFERROR(I13/H13*1000,0)</f>
         <v>0</v>
       </c>
-      <c r="K13" s="24">
+      <c r="K13" s="21">
         <f>E13+I13</f>
         <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>August 2026</t>
         </is>
@@ -1038,24 +1061,24 @@
       <c r="C14" s="14" t="n"/>
       <c r="D14" s="14" t="n"/>
       <c r="E14" s="19" t="n"/>
-      <c r="F14" s="20">
+      <c r="F14" s="23">
         <f>IFERROR(E14/D14*1000,0)</f>
         <v>0</v>
       </c>
       <c r="G14" s="16" t="n"/>
       <c r="H14" s="14" t="n"/>
       <c r="I14" s="19" t="n"/>
-      <c r="J14" s="20">
+      <c r="J14" s="23">
         <f>IFERROR(I14/H14*1000,0)</f>
         <v>0</v>
       </c>
-      <c r="K14" s="21">
+      <c r="K14" s="24">
         <f>E14+I14</f>
         <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="22" t="inlineStr">
+      <c r="A15" s="18" t="inlineStr">
         <is>
           <t>September 2026</t>
         </is>
@@ -1064,24 +1087,24 @@
       <c r="C15" s="14" t="n"/>
       <c r="D15" s="14" t="n"/>
       <c r="E15" s="19" t="n"/>
-      <c r="F15" s="23">
+      <c r="F15" s="20">
         <f>IFERROR(E15/D15*1000,0)</f>
         <v>0</v>
       </c>
       <c r="G15" s="16" t="n"/>
       <c r="H15" s="14" t="n"/>
       <c r="I15" s="19" t="n"/>
-      <c r="J15" s="23">
+      <c r="J15" s="20">
         <f>IFERROR(I15/H15*1000,0)</f>
         <v>0</v>
       </c>
-      <c r="K15" s="24">
+      <c r="K15" s="21">
         <f>E15+I15</f>
         <v>0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="inlineStr">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>October 2026</t>
         </is>
@@ -1090,24 +1113,24 @@
       <c r="C16" s="14" t="n"/>
       <c r="D16" s="14" t="n"/>
       <c r="E16" s="19" t="n"/>
-      <c r="F16" s="20">
+      <c r="F16" s="23">
         <f>IFERROR(E16/D16*1000,0)</f>
         <v>0</v>
       </c>
       <c r="G16" s="16" t="n"/>
       <c r="H16" s="14" t="n"/>
       <c r="I16" s="19" t="n"/>
-      <c r="J16" s="20">
+      <c r="J16" s="23">
         <f>IFERROR(I16/H16*1000,0)</f>
         <v>0</v>
       </c>
-      <c r="K16" s="21">
+      <c r="K16" s="24">
         <f>E16+I16</f>
         <v>0</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="22" t="inlineStr">
+      <c r="A17" s="18" t="inlineStr">
         <is>
           <t>November 2026</t>
         </is>
@@ -1116,24 +1139,24 @@
       <c r="C17" s="14" t="n"/>
       <c r="D17" s="14" t="n"/>
       <c r="E17" s="19" t="n"/>
-      <c r="F17" s="23">
+      <c r="F17" s="20">
         <f>IFERROR(E17/D17*1000,0)</f>
         <v>0</v>
       </c>
       <c r="G17" s="16" t="n"/>
       <c r="H17" s="14" t="n"/>
       <c r="I17" s="19" t="n"/>
-      <c r="J17" s="23">
+      <c r="J17" s="20">
         <f>IFERROR(I17/H17*1000,0)</f>
         <v>0</v>
       </c>
-      <c r="K17" s="24">
+      <c r="K17" s="21">
         <f>E17+I17</f>
         <v>0</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="18" t="inlineStr">
+      <c r="A18" s="22" t="inlineStr">
         <is>
           <t>December 2026</t>
         </is>
@@ -1142,24 +1165,24 @@
       <c r="C18" s="14" t="n"/>
       <c r="D18" s="14" t="n"/>
       <c r="E18" s="19" t="n"/>
-      <c r="F18" s="20">
+      <c r="F18" s="23">
         <f>IFERROR(E18/D18*1000,0)</f>
         <v>0</v>
       </c>
       <c r="G18" s="16" t="n"/>
       <c r="H18" s="14" t="n"/>
       <c r="I18" s="19" t="n"/>
-      <c r="J18" s="20">
+      <c r="J18" s="23">
         <f>IFERROR(I18/H18*1000,0)</f>
         <v>0</v>
       </c>
-      <c r="K18" s="21">
+      <c r="K18" s="24">
         <f>E18+I18</f>
         <v>0</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="22" t="inlineStr">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>January 2027</t>
         </is>
@@ -1168,24 +1191,24 @@
       <c r="C19" s="14" t="n"/>
       <c r="D19" s="14" t="n"/>
       <c r="E19" s="19" t="n"/>
-      <c r="F19" s="23">
+      <c r="F19" s="20">
         <f>IFERROR(E19/D19*1000,0)</f>
         <v>0</v>
       </c>
       <c r="G19" s="16" t="n"/>
       <c r="H19" s="14" t="n"/>
       <c r="I19" s="19" t="n"/>
-      <c r="J19" s="23">
+      <c r="J19" s="20">
         <f>IFERROR(I19/H19*1000,0)</f>
         <v>0</v>
       </c>
-      <c r="K19" s="24">
+      <c r="K19" s="21">
         <f>E19+I19</f>
         <v>0</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="18" t="inlineStr">
+      <c r="A20" s="22" t="inlineStr">
         <is>
           <t>February 2027</t>
         </is>
@@ -1194,24 +1217,24 @@
       <c r="C20" s="14" t="n"/>
       <c r="D20" s="14" t="n"/>
       <c r="E20" s="19" t="n"/>
-      <c r="F20" s="20">
+      <c r="F20" s="23">
         <f>IFERROR(E20/D20*1000,0)</f>
         <v>0</v>
       </c>
       <c r="G20" s="16" t="n"/>
       <c r="H20" s="14" t="n"/>
       <c r="I20" s="19" t="n"/>
-      <c r="J20" s="20">
+      <c r="J20" s="23">
         <f>IFERROR(I20/H20*1000,0)</f>
         <v>0</v>
       </c>
-      <c r="K20" s="21">
+      <c r="K20" s="24">
         <f>E20+I20</f>
         <v>0</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="22" t="inlineStr">
+      <c r="A21" s="18" t="inlineStr">
         <is>
           <t>March 2027</t>
         </is>
@@ -1220,18 +1243,18 @@
       <c r="C21" s="14" t="n"/>
       <c r="D21" s="14" t="n"/>
       <c r="E21" s="19" t="n"/>
-      <c r="F21" s="23">
+      <c r="F21" s="20">
         <f>IFERROR(E21/D21*1000,0)</f>
         <v>0</v>
       </c>
       <c r="G21" s="16" t="n"/>
       <c r="H21" s="14" t="n"/>
       <c r="I21" s="19" t="n"/>
-      <c r="J21" s="23">
+      <c r="J21" s="20">
         <f>IFERROR(I21/H21*1000,0)</f>
         <v>0</v>
       </c>
-      <c r="K21" s="24">
+      <c r="K21" s="21">
         <f>E21+I21</f>
         <v>0</v>
       </c>
@@ -1278,7 +1301,7 @@
       <c r="J25" s="29" t="n"/>
       <c r="K25" s="30">
         <f>SUM(B8:B21)</f>
-        <v>15</v>
+        <v>84</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
@@ -1298,7 +1321,7 @@
       <c r="J26" s="29" t="n"/>
       <c r="K26" s="30">
         <f>SUM(C8:C21)</f>
-        <v>1100000</v>
+        <v>14300000</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
@@ -1317,8 +1340,8 @@
       <c r="I27" s="29" t="n"/>
       <c r="J27" s="29" t="n"/>
       <c r="K27" s="30">
-        <f>SUM(D12:D21)</f>
-        <v>606700</v>
+        <f>SUM(D11:D21)</f>
+        <v>650000</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
@@ -1337,8 +1360,8 @@
       <c r="I28" s="29" t="n"/>
       <c r="J28" s="29" t="n"/>
       <c r="K28" s="31">
-        <f>SUM(E12:E21)</f>
-        <v>146.81</v>
+        <f>SUM(E11:E21)</f>
+        <v>157.66</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
@@ -1358,7 +1381,7 @@
       <c r="J29" s="29" t="n"/>
       <c r="K29" s="32">
         <f>IFERROR(K28/K27*1000,0)</f>
-        <v>0.24198120982363605</v>
+        <v>0.24255384615384618</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
@@ -1395,7 +1418,7 @@
       <c r="J31" s="29" t="n"/>
       <c r="K31" s="30">
         <f>SUM(G8:G21)</f>
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
@@ -1414,8 +1437,8 @@
       <c r="I32" s="29" t="n"/>
       <c r="J32" s="29" t="n"/>
       <c r="K32" s="30">
-        <f>SUM(H12:H21)</f>
-        <v>31600</v>
+        <f>SUM(H11:H21)</f>
+        <v>38000</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
@@ -1434,8 +1457,8 @@
       <c r="I33" s="29" t="n"/>
       <c r="J33" s="29" t="n"/>
       <c r="K33" s="31">
-        <f>SUM(I12:I21)</f>
-        <v>59.84</v>
+        <f>SUM(I11:I21)</f>
+        <v>66.26</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
@@ -1455,7 +1478,7 @@
       <c r="J34" s="29" t="n"/>
       <c r="K34" s="32">
         <f>IFERROR(K33/K32*1000,0)</f>
-        <v>1.8936708860759495</v>
+        <v>1.743684210526316</v>
       </c>
     </row>
     <row r="36" ht="26" customHeight="1">
@@ -1475,13 +1498,13 @@
       <c r="J36" s="35" t="n"/>
       <c r="K36" s="36">
         <f>SUM(K8:K21)</f>
-        <v>206.65</v>
+        <v>223.92000000000002</v>
       </c>
     </row>
     <row r="38" ht="56" customHeight="1">
       <c r="A38" s="37" t="inlineStr">
         <is>
-          <t>Note: February–May 2026 are shaded gray because the channel wasn't monetized yet — Videos/Shorts Published and Views can still be logged, but Engaged Views, Earnings and RPM are marked N/A and excluded from every earnings/RPM total below. Monetized tracking begins June 2026, filled in with your real reported numbers (Shorts $146.81 + Long-Form $59.84 = $206.65). Shorts RPM is calculated on Engaged Views; Long-Form RPM is calculated on total Long Views, since every long-form view is monetized. Enter your real figures for the remaining months as they happen.</t>
+          <t>Note: February–April 2026 are shaded gray because the channel wasn't monetized yet — Videos/Shorts Published and Views can still be logged, but Engaged Views, Earnings and RPM are marked N/A and excluded from every earnings/RPM total below. Monetized tracking begins May 2026, filled in with your real reported numbers (Shorts $10.85 + Long-Form $6.42 = $17.27), continuing with June 2026 (Shorts $146.81 + Long-Form $59.84 = $206.65). Shorts RPM is calculated on Engaged Views; Long-Form RPM is calculated on total Long Views, since every long-form view is monetized. Enter your real figures for the remaining months as they happen.</t>
         </is>
       </c>
     </row>

</xml_diff>